<commit_message>
modified python scripts and more routes added
</commit_message>
<xml_diff>
--- a/backend/data-filtering/stops_table.xlsx
+++ b/backend/data-filtering/stops_table.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\travel\backend\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\travel\backend\data-filtering\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D5B24ED-1DE4-4245-8770-78C6D8F4A39D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FC8416C-F8E5-468C-981B-7FED838B7EC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{0946D8EF-606D-4B7F-92DD-E4F456A214B3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{0946D8EF-606D-4B7F-92DD-E4F456A214B3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>